<commit_message>
Fix empty task list in detail sheet caused by Excel implicit intersection
Excel 365 prepends @ (implicit intersection) to formulas in files
written by external tools, which broke the AGGREGATE array formula
in the detail sheet's helper column and left the task table blank.

Replace the array approach with a lookup-key scheme that uses no
array semantics at all:
- 작업 sheet gets a hidden helper column N building the key
  "프로젝트ID|n번째" via a running COUNTIF
- 프로젝트 상세 helper column finds each task with a plain MATCH
  on that key

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BSNoKB9xi2beynDHXB1bmC
</commit_message>
<xml_diff>
--- a/프로젝트_트랙커.xlsx
+++ b/프로젝트_트랙커.xlsx
@@ -3618,7 +3618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L105"/>
+  <dimension ref="B2:N105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3633,6 +3633,7 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -3751,6 +3752,10 @@
         <v/>
       </c>
       <c r="L6" s="39" t="inlineStr"/>
+      <c r="N6">
+        <f>IF($B6="","",$C6&amp;"|"&amp;COUNTIF($C$6:$C6,$C6))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="24" t="inlineStr">
@@ -3797,6 +3802,10 @@
         <v/>
       </c>
       <c r="L7" s="39" t="inlineStr"/>
+      <c r="N7">
+        <f>IF($B7="","",$C7&amp;"|"&amp;COUNTIF($C$6:$C7,$C7))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="24" t="inlineStr">
@@ -3843,6 +3852,10 @@
         <v/>
       </c>
       <c r="L8" s="39" t="inlineStr"/>
+      <c r="N8">
+        <f>IF($B8="","",$C8&amp;"|"&amp;COUNTIF($C$6:$C8,$C8))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="24" t="inlineStr">
@@ -3889,6 +3902,10 @@
         <v/>
       </c>
       <c r="L9" s="39" t="inlineStr"/>
+      <c r="N9">
+        <f>IF($B9="","",$C9&amp;"|"&amp;COUNTIF($C$6:$C9,$C9))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="24" t="inlineStr">
@@ -3939,6 +3956,10 @@
           <t>심사 기간 고려</t>
         </is>
       </c>
+      <c r="N10">
+        <f>IF($B10="","",$C10&amp;"|"&amp;COUNTIF($C$6:$C10,$C10))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="24" t="inlineStr">
@@ -3988,6 +4009,10 @@
         <is>
           <t>외주사 회신 대기</t>
         </is>
+      </c>
+      <c r="N11">
+        <f>IF($B11="","",$C11&amp;"|"&amp;COUNTIF($C$6:$C11,$C11))</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -4005,6 +4030,10 @@
         <v/>
       </c>
       <c r="L12" s="39" t="n"/>
+      <c r="N12">
+        <f>IF($B12="","",$C12&amp;"|"&amp;COUNTIF($C$6:$C12,$C12))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="24" t="n"/>
@@ -4021,6 +4050,10 @@
         <v/>
       </c>
       <c r="L13" s="39" t="n"/>
+      <c r="N13">
+        <f>IF($B13="","",$C13&amp;"|"&amp;COUNTIF($C$6:$C13,$C13))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="24" t="n"/>
@@ -4037,6 +4070,10 @@
         <v/>
       </c>
       <c r="L14" s="39" t="n"/>
+      <c r="N14">
+        <f>IF($B14="","",$C14&amp;"|"&amp;COUNTIF($C$6:$C14,$C14))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="24" t="n"/>
@@ -4053,6 +4090,10 @@
         <v/>
       </c>
       <c r="L15" s="39" t="n"/>
+      <c r="N15">
+        <f>IF($B15="","",$C15&amp;"|"&amp;COUNTIF($C$6:$C15,$C15))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="24" t="n"/>
@@ -4069,6 +4110,10 @@
         <v/>
       </c>
       <c r="L16" s="39" t="n"/>
+      <c r="N16">
+        <f>IF($B16="","",$C16&amp;"|"&amp;COUNTIF($C$6:$C16,$C16))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="24" t="n"/>
@@ -4085,6 +4130,10 @@
         <v/>
       </c>
       <c r="L17" s="39" t="n"/>
+      <c r="N17">
+        <f>IF($B17="","",$C17&amp;"|"&amp;COUNTIF($C$6:$C17,$C17))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="24" t="n"/>
@@ -4101,6 +4150,10 @@
         <v/>
       </c>
       <c r="L18" s="39" t="n"/>
+      <c r="N18">
+        <f>IF($B18="","",$C18&amp;"|"&amp;COUNTIF($C$6:$C18,$C18))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="24" t="n"/>
@@ -4117,6 +4170,10 @@
         <v/>
       </c>
       <c r="L19" s="39" t="n"/>
+      <c r="N19">
+        <f>IF($B19="","",$C19&amp;"|"&amp;COUNTIF($C$6:$C19,$C19))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="24" t="n"/>
@@ -4133,6 +4190,10 @@
         <v/>
       </c>
       <c r="L20" s="39" t="n"/>
+      <c r="N20">
+        <f>IF($B20="","",$C20&amp;"|"&amp;COUNTIF($C$6:$C20,$C20))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="24" t="n"/>
@@ -4149,6 +4210,10 @@
         <v/>
       </c>
       <c r="L21" s="39" t="n"/>
+      <c r="N21">
+        <f>IF($B21="","",$C21&amp;"|"&amp;COUNTIF($C$6:$C21,$C21))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="24" t="n"/>
@@ -4165,6 +4230,10 @@
         <v/>
       </c>
       <c r="L22" s="39" t="n"/>
+      <c r="N22">
+        <f>IF($B22="","",$C22&amp;"|"&amp;COUNTIF($C$6:$C22,$C22))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="24" t="n"/>
@@ -4181,6 +4250,10 @@
         <v/>
       </c>
       <c r="L23" s="39" t="n"/>
+      <c r="N23">
+        <f>IF($B23="","",$C23&amp;"|"&amp;COUNTIF($C$6:$C23,$C23))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="24" t="n"/>
@@ -4197,6 +4270,10 @@
         <v/>
       </c>
       <c r="L24" s="39" t="n"/>
+      <c r="N24">
+        <f>IF($B24="","",$C24&amp;"|"&amp;COUNTIF($C$6:$C24,$C24))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="24" t="n"/>
@@ -4213,6 +4290,10 @@
         <v/>
       </c>
       <c r="L25" s="39" t="n"/>
+      <c r="N25">
+        <f>IF($B25="","",$C25&amp;"|"&amp;COUNTIF($C$6:$C25,$C25))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="24" t="n"/>
@@ -4229,6 +4310,10 @@
         <v/>
       </c>
       <c r="L26" s="39" t="n"/>
+      <c r="N26">
+        <f>IF($B26="","",$C26&amp;"|"&amp;COUNTIF($C$6:$C26,$C26))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="24" t="n"/>
@@ -4245,6 +4330,10 @@
         <v/>
       </c>
       <c r="L27" s="39" t="n"/>
+      <c r="N27">
+        <f>IF($B27="","",$C27&amp;"|"&amp;COUNTIF($C$6:$C27,$C27))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="24" t="n"/>
@@ -4261,6 +4350,10 @@
         <v/>
       </c>
       <c r="L28" s="39" t="n"/>
+      <c r="N28">
+        <f>IF($B28="","",$C28&amp;"|"&amp;COUNTIF($C$6:$C28,$C28))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="24" t="n"/>
@@ -4277,6 +4370,10 @@
         <v/>
       </c>
       <c r="L29" s="39" t="n"/>
+      <c r="N29">
+        <f>IF($B29="","",$C29&amp;"|"&amp;COUNTIF($C$6:$C29,$C29))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="24" t="n"/>
@@ -4293,6 +4390,10 @@
         <v/>
       </c>
       <c r="L30" s="39" t="n"/>
+      <c r="N30">
+        <f>IF($B30="","",$C30&amp;"|"&amp;COUNTIF($C$6:$C30,$C30))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="24" t="n"/>
@@ -4309,6 +4410,10 @@
         <v/>
       </c>
       <c r="L31" s="39" t="n"/>
+      <c r="N31">
+        <f>IF($B31="","",$C31&amp;"|"&amp;COUNTIF($C$6:$C31,$C31))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="24" t="n"/>
@@ -4325,6 +4430,10 @@
         <v/>
       </c>
       <c r="L32" s="39" t="n"/>
+      <c r="N32">
+        <f>IF($B32="","",$C32&amp;"|"&amp;COUNTIF($C$6:$C32,$C32))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="24" t="n"/>
@@ -4341,6 +4450,10 @@
         <v/>
       </c>
       <c r="L33" s="39" t="n"/>
+      <c r="N33">
+        <f>IF($B33="","",$C33&amp;"|"&amp;COUNTIF($C$6:$C33,$C33))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="24" t="n"/>
@@ -4357,6 +4470,10 @@
         <v/>
       </c>
       <c r="L34" s="39" t="n"/>
+      <c r="N34">
+        <f>IF($B34="","",$C34&amp;"|"&amp;COUNTIF($C$6:$C34,$C34))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="24" t="n"/>
@@ -4373,6 +4490,10 @@
         <v/>
       </c>
       <c r="L35" s="39" t="n"/>
+      <c r="N35">
+        <f>IF($B35="","",$C35&amp;"|"&amp;COUNTIF($C$6:$C35,$C35))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="24" t="n"/>
@@ -4389,6 +4510,10 @@
         <v/>
       </c>
       <c r="L36" s="39" t="n"/>
+      <c r="N36">
+        <f>IF($B36="","",$C36&amp;"|"&amp;COUNTIF($C$6:$C36,$C36))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="24" t="n"/>
@@ -4405,6 +4530,10 @@
         <v/>
       </c>
       <c r="L37" s="39" t="n"/>
+      <c r="N37">
+        <f>IF($B37="","",$C37&amp;"|"&amp;COUNTIF($C$6:$C37,$C37))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="24" t="n"/>
@@ -4421,6 +4550,10 @@
         <v/>
       </c>
       <c r="L38" s="39" t="n"/>
+      <c r="N38">
+        <f>IF($B38="","",$C38&amp;"|"&amp;COUNTIF($C$6:$C38,$C38))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="24" t="n"/>
@@ -4437,6 +4570,10 @@
         <v/>
       </c>
       <c r="L39" s="39" t="n"/>
+      <c r="N39">
+        <f>IF($B39="","",$C39&amp;"|"&amp;COUNTIF($C$6:$C39,$C39))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="24" t="n"/>
@@ -4453,6 +4590,10 @@
         <v/>
       </c>
       <c r="L40" s="39" t="n"/>
+      <c r="N40">
+        <f>IF($B40="","",$C40&amp;"|"&amp;COUNTIF($C$6:$C40,$C40))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="24" t="n"/>
@@ -4469,6 +4610,10 @@
         <v/>
       </c>
       <c r="L41" s="39" t="n"/>
+      <c r="N41">
+        <f>IF($B41="","",$C41&amp;"|"&amp;COUNTIF($C$6:$C41,$C41))</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="24" t="n"/>
@@ -4485,6 +4630,10 @@
         <v/>
       </c>
       <c r="L42" s="39" t="n"/>
+      <c r="N42">
+        <f>IF($B42="","",$C42&amp;"|"&amp;COUNTIF($C$6:$C42,$C42))</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="24" t="n"/>
@@ -4501,6 +4650,10 @@
         <v/>
       </c>
       <c r="L43" s="39" t="n"/>
+      <c r="N43">
+        <f>IF($B43="","",$C43&amp;"|"&amp;COUNTIF($C$6:$C43,$C43))</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="24" t="n"/>
@@ -4517,6 +4670,10 @@
         <v/>
       </c>
       <c r="L44" s="39" t="n"/>
+      <c r="N44">
+        <f>IF($B44="","",$C44&amp;"|"&amp;COUNTIF($C$6:$C44,$C44))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="24" t="n"/>
@@ -4533,6 +4690,10 @@
         <v/>
       </c>
       <c r="L45" s="39" t="n"/>
+      <c r="N45">
+        <f>IF($B45="","",$C45&amp;"|"&amp;COUNTIF($C$6:$C45,$C45))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="24" t="n"/>
@@ -4549,6 +4710,10 @@
         <v/>
       </c>
       <c r="L46" s="39" t="n"/>
+      <c r="N46">
+        <f>IF($B46="","",$C46&amp;"|"&amp;COUNTIF($C$6:$C46,$C46))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="24" t="n"/>
@@ -4565,6 +4730,10 @@
         <v/>
       </c>
       <c r="L47" s="39" t="n"/>
+      <c r="N47">
+        <f>IF($B47="","",$C47&amp;"|"&amp;COUNTIF($C$6:$C47,$C47))</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="24" t="n"/>
@@ -4581,6 +4750,10 @@
         <v/>
       </c>
       <c r="L48" s="39" t="n"/>
+      <c r="N48">
+        <f>IF($B48="","",$C48&amp;"|"&amp;COUNTIF($C$6:$C48,$C48))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="24" t="n"/>
@@ -4597,6 +4770,10 @@
         <v/>
       </c>
       <c r="L49" s="39" t="n"/>
+      <c r="N49">
+        <f>IF($B49="","",$C49&amp;"|"&amp;COUNTIF($C$6:$C49,$C49))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="24" t="n"/>
@@ -4613,6 +4790,10 @@
         <v/>
       </c>
       <c r="L50" s="39" t="n"/>
+      <c r="N50">
+        <f>IF($B50="","",$C50&amp;"|"&amp;COUNTIF($C$6:$C50,$C50))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="24" t="n"/>
@@ -4629,6 +4810,10 @@
         <v/>
       </c>
       <c r="L51" s="39" t="n"/>
+      <c r="N51">
+        <f>IF($B51="","",$C51&amp;"|"&amp;COUNTIF($C$6:$C51,$C51))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="24" t="n"/>
@@ -4645,6 +4830,10 @@
         <v/>
       </c>
       <c r="L52" s="39" t="n"/>
+      <c r="N52">
+        <f>IF($B52="","",$C52&amp;"|"&amp;COUNTIF($C$6:$C52,$C52))</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="24" t="n"/>
@@ -4661,6 +4850,10 @@
         <v/>
       </c>
       <c r="L53" s="39" t="n"/>
+      <c r="N53">
+        <f>IF($B53="","",$C53&amp;"|"&amp;COUNTIF($C$6:$C53,$C53))</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="24" t="n"/>
@@ -4677,6 +4870,10 @@
         <v/>
       </c>
       <c r="L54" s="39" t="n"/>
+      <c r="N54">
+        <f>IF($B54="","",$C54&amp;"|"&amp;COUNTIF($C$6:$C54,$C54))</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="24" t="n"/>
@@ -4693,6 +4890,10 @@
         <v/>
       </c>
       <c r="L55" s="39" t="n"/>
+      <c r="N55">
+        <f>IF($B55="","",$C55&amp;"|"&amp;COUNTIF($C$6:$C55,$C55))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="24" t="n"/>
@@ -4709,6 +4910,10 @@
         <v/>
       </c>
       <c r="L56" s="39" t="n"/>
+      <c r="N56">
+        <f>IF($B56="","",$C56&amp;"|"&amp;COUNTIF($C$6:$C56,$C56))</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="24" t="n"/>
@@ -4725,6 +4930,10 @@
         <v/>
       </c>
       <c r="L57" s="39" t="n"/>
+      <c r="N57">
+        <f>IF($B57="","",$C57&amp;"|"&amp;COUNTIF($C$6:$C57,$C57))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="24" t="n"/>
@@ -4741,6 +4950,10 @@
         <v/>
       </c>
       <c r="L58" s="39" t="n"/>
+      <c r="N58">
+        <f>IF($B58="","",$C58&amp;"|"&amp;COUNTIF($C$6:$C58,$C58))</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="B59" s="24" t="n"/>
@@ -4757,6 +4970,10 @@
         <v/>
       </c>
       <c r="L59" s="39" t="n"/>
+      <c r="N59">
+        <f>IF($B59="","",$C59&amp;"|"&amp;COUNTIF($C$6:$C59,$C59))</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="24" t="n"/>
@@ -4773,6 +4990,10 @@
         <v/>
       </c>
       <c r="L60" s="39" t="n"/>
+      <c r="N60">
+        <f>IF($B60="","",$C60&amp;"|"&amp;COUNTIF($C$6:$C60,$C60))</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="24" t="n"/>
@@ -4789,6 +5010,10 @@
         <v/>
       </c>
       <c r="L61" s="39" t="n"/>
+      <c r="N61">
+        <f>IF($B61="","",$C61&amp;"|"&amp;COUNTIF($C$6:$C61,$C61))</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="24" t="n"/>
@@ -4805,6 +5030,10 @@
         <v/>
       </c>
       <c r="L62" s="39" t="n"/>
+      <c r="N62">
+        <f>IF($B62="","",$C62&amp;"|"&amp;COUNTIF($C$6:$C62,$C62))</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="24" t="n"/>
@@ -4821,6 +5050,10 @@
         <v/>
       </c>
       <c r="L63" s="39" t="n"/>
+      <c r="N63">
+        <f>IF($B63="","",$C63&amp;"|"&amp;COUNTIF($C$6:$C63,$C63))</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="B64" s="24" t="n"/>
@@ -4837,6 +5070,10 @@
         <v/>
       </c>
       <c r="L64" s="39" t="n"/>
+      <c r="N64">
+        <f>IF($B64="","",$C64&amp;"|"&amp;COUNTIF($C$6:$C64,$C64))</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="24" t="n"/>
@@ -4853,6 +5090,10 @@
         <v/>
       </c>
       <c r="L65" s="39" t="n"/>
+      <c r="N65">
+        <f>IF($B65="","",$C65&amp;"|"&amp;COUNTIF($C$6:$C65,$C65))</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="B66" s="24" t="n"/>
@@ -4869,6 +5110,10 @@
         <v/>
       </c>
       <c r="L66" s="39" t="n"/>
+      <c r="N66">
+        <f>IF($B66="","",$C66&amp;"|"&amp;COUNTIF($C$6:$C66,$C66))</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="B67" s="24" t="n"/>
@@ -4885,6 +5130,10 @@
         <v/>
       </c>
       <c r="L67" s="39" t="n"/>
+      <c r="N67">
+        <f>IF($B67="","",$C67&amp;"|"&amp;COUNTIF($C$6:$C67,$C67))</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="24" t="n"/>
@@ -4901,6 +5150,10 @@
         <v/>
       </c>
       <c r="L68" s="39" t="n"/>
+      <c r="N68">
+        <f>IF($B68="","",$C68&amp;"|"&amp;COUNTIF($C$6:$C68,$C68))</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="24" t="n"/>
@@ -4917,6 +5170,10 @@
         <v/>
       </c>
       <c r="L69" s="39" t="n"/>
+      <c r="N69">
+        <f>IF($B69="","",$C69&amp;"|"&amp;COUNTIF($C$6:$C69,$C69))</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="B70" s="24" t="n"/>
@@ -4933,6 +5190,10 @@
         <v/>
       </c>
       <c r="L70" s="39" t="n"/>
+      <c r="N70">
+        <f>IF($B70="","",$C70&amp;"|"&amp;COUNTIF($C$6:$C70,$C70))</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="B71" s="24" t="n"/>
@@ -4949,6 +5210,10 @@
         <v/>
       </c>
       <c r="L71" s="39" t="n"/>
+      <c r="N71">
+        <f>IF($B71="","",$C71&amp;"|"&amp;COUNTIF($C$6:$C71,$C71))</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="24" t="n"/>
@@ -4965,6 +5230,10 @@
         <v/>
       </c>
       <c r="L72" s="39" t="n"/>
+      <c r="N72">
+        <f>IF($B72="","",$C72&amp;"|"&amp;COUNTIF($C$6:$C72,$C72))</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="B73" s="24" t="n"/>
@@ -4981,6 +5250,10 @@
         <v/>
       </c>
       <c r="L73" s="39" t="n"/>
+      <c r="N73">
+        <f>IF($B73="","",$C73&amp;"|"&amp;COUNTIF($C$6:$C73,$C73))</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="B74" s="24" t="n"/>
@@ -4997,6 +5270,10 @@
         <v/>
       </c>
       <c r="L74" s="39" t="n"/>
+      <c r="N74">
+        <f>IF($B74="","",$C74&amp;"|"&amp;COUNTIF($C$6:$C74,$C74))</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="B75" s="24" t="n"/>
@@ -5013,6 +5290,10 @@
         <v/>
       </c>
       <c r="L75" s="39" t="n"/>
+      <c r="N75">
+        <f>IF($B75="","",$C75&amp;"|"&amp;COUNTIF($C$6:$C75,$C75))</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="B76" s="24" t="n"/>
@@ -5029,6 +5310,10 @@
         <v/>
       </c>
       <c r="L76" s="39" t="n"/>
+      <c r="N76">
+        <f>IF($B76="","",$C76&amp;"|"&amp;COUNTIF($C$6:$C76,$C76))</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="24" t="n"/>
@@ -5045,6 +5330,10 @@
         <v/>
       </c>
       <c r="L77" s="39" t="n"/>
+      <c r="N77">
+        <f>IF($B77="","",$C77&amp;"|"&amp;COUNTIF($C$6:$C77,$C77))</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="24" t="n"/>
@@ -5061,6 +5350,10 @@
         <v/>
       </c>
       <c r="L78" s="39" t="n"/>
+      <c r="N78">
+        <f>IF($B78="","",$C78&amp;"|"&amp;COUNTIF($C$6:$C78,$C78))</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="24" t="n"/>
@@ -5077,6 +5370,10 @@
         <v/>
       </c>
       <c r="L79" s="39" t="n"/>
+      <c r="N79">
+        <f>IF($B79="","",$C79&amp;"|"&amp;COUNTIF($C$6:$C79,$C79))</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="24" t="n"/>
@@ -5093,6 +5390,10 @@
         <v/>
       </c>
       <c r="L80" s="39" t="n"/>
+      <c r="N80">
+        <f>IF($B80="","",$C80&amp;"|"&amp;COUNTIF($C$6:$C80,$C80))</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="24" t="n"/>
@@ -5109,6 +5410,10 @@
         <v/>
       </c>
       <c r="L81" s="39" t="n"/>
+      <c r="N81">
+        <f>IF($B81="","",$C81&amp;"|"&amp;COUNTIF($C$6:$C81,$C81))</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="B82" s="24" t="n"/>
@@ -5125,6 +5430,10 @@
         <v/>
       </c>
       <c r="L82" s="39" t="n"/>
+      <c r="N82">
+        <f>IF($B82="","",$C82&amp;"|"&amp;COUNTIF($C$6:$C82,$C82))</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="B83" s="24" t="n"/>
@@ -5141,6 +5450,10 @@
         <v/>
       </c>
       <c r="L83" s="39" t="n"/>
+      <c r="N83">
+        <f>IF($B83="","",$C83&amp;"|"&amp;COUNTIF($C$6:$C83,$C83))</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="B84" s="24" t="n"/>
@@ -5157,6 +5470,10 @@
         <v/>
       </c>
       <c r="L84" s="39" t="n"/>
+      <c r="N84">
+        <f>IF($B84="","",$C84&amp;"|"&amp;COUNTIF($C$6:$C84,$C84))</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="24" t="n"/>
@@ -5173,6 +5490,10 @@
         <v/>
       </c>
       <c r="L85" s="39" t="n"/>
+      <c r="N85">
+        <f>IF($B85="","",$C85&amp;"|"&amp;COUNTIF($C$6:$C85,$C85))</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="B86" s="24" t="n"/>
@@ -5189,6 +5510,10 @@
         <v/>
       </c>
       <c r="L86" s="39" t="n"/>
+      <c r="N86">
+        <f>IF($B86="","",$C86&amp;"|"&amp;COUNTIF($C$6:$C86,$C86))</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="24" t="n"/>
@@ -5205,6 +5530,10 @@
         <v/>
       </c>
       <c r="L87" s="39" t="n"/>
+      <c r="N87">
+        <f>IF($B87="","",$C87&amp;"|"&amp;COUNTIF($C$6:$C87,$C87))</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="B88" s="24" t="n"/>
@@ -5221,6 +5550,10 @@
         <v/>
       </c>
       <c r="L88" s="39" t="n"/>
+      <c r="N88">
+        <f>IF($B88="","",$C88&amp;"|"&amp;COUNTIF($C$6:$C88,$C88))</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="24" t="n"/>
@@ -5237,6 +5570,10 @@
         <v/>
       </c>
       <c r="L89" s="39" t="n"/>
+      <c r="N89">
+        <f>IF($B89="","",$C89&amp;"|"&amp;COUNTIF($C$6:$C89,$C89))</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="B90" s="24" t="n"/>
@@ -5253,6 +5590,10 @@
         <v/>
       </c>
       <c r="L90" s="39" t="n"/>
+      <c r="N90">
+        <f>IF($B90="","",$C90&amp;"|"&amp;COUNTIF($C$6:$C90,$C90))</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="B91" s="24" t="n"/>
@@ -5269,6 +5610,10 @@
         <v/>
       </c>
       <c r="L91" s="39" t="n"/>
+      <c r="N91">
+        <f>IF($B91="","",$C91&amp;"|"&amp;COUNTIF($C$6:$C91,$C91))</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="24" t="n"/>
@@ -5285,6 +5630,10 @@
         <v/>
       </c>
       <c r="L92" s="39" t="n"/>
+      <c r="N92">
+        <f>IF($B92="","",$C92&amp;"|"&amp;COUNTIF($C$6:$C92,$C92))</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="24" t="n"/>
@@ -5301,6 +5650,10 @@
         <v/>
       </c>
       <c r="L93" s="39" t="n"/>
+      <c r="N93">
+        <f>IF($B93="","",$C93&amp;"|"&amp;COUNTIF($C$6:$C93,$C93))</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="24" t="n"/>
@@ -5317,6 +5670,10 @@
         <v/>
       </c>
       <c r="L94" s="39" t="n"/>
+      <c r="N94">
+        <f>IF($B94="","",$C94&amp;"|"&amp;COUNTIF($C$6:$C94,$C94))</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="24" t="n"/>
@@ -5333,6 +5690,10 @@
         <v/>
       </c>
       <c r="L95" s="39" t="n"/>
+      <c r="N95">
+        <f>IF($B95="","",$C95&amp;"|"&amp;COUNTIF($C$6:$C95,$C95))</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="24" t="n"/>
@@ -5349,6 +5710,10 @@
         <v/>
       </c>
       <c r="L96" s="39" t="n"/>
+      <c r="N96">
+        <f>IF($B96="","",$C96&amp;"|"&amp;COUNTIF($C$6:$C96,$C96))</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="B97" s="24" t="n"/>
@@ -5365,6 +5730,10 @@
         <v/>
       </c>
       <c r="L97" s="39" t="n"/>
+      <c r="N97">
+        <f>IF($B97="","",$C97&amp;"|"&amp;COUNTIF($C$6:$C97,$C97))</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="B98" s="24" t="n"/>
@@ -5381,6 +5750,10 @@
         <v/>
       </c>
       <c r="L98" s="39" t="n"/>
+      <c r="N98">
+        <f>IF($B98="","",$C98&amp;"|"&amp;COUNTIF($C$6:$C98,$C98))</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="24" t="n"/>
@@ -5397,6 +5770,10 @@
         <v/>
       </c>
       <c r="L99" s="39" t="n"/>
+      <c r="N99">
+        <f>IF($B99="","",$C99&amp;"|"&amp;COUNTIF($C$6:$C99,$C99))</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="24" t="n"/>
@@ -5413,6 +5790,10 @@
         <v/>
       </c>
       <c r="L100" s="39" t="n"/>
+      <c r="N100">
+        <f>IF($B100="","",$C100&amp;"|"&amp;COUNTIF($C$6:$C100,$C100))</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="B101" s="24" t="n"/>
@@ -5429,6 +5810,10 @@
         <v/>
       </c>
       <c r="L101" s="39" t="n"/>
+      <c r="N101">
+        <f>IF($B101="","",$C101&amp;"|"&amp;COUNTIF($C$6:$C101,$C101))</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="B102" s="24" t="n"/>
@@ -5445,6 +5830,10 @@
         <v/>
       </c>
       <c r="L102" s="39" t="n"/>
+      <c r="N102">
+        <f>IF($B102="","",$C102&amp;"|"&amp;COUNTIF($C$6:$C102,$C102))</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="B103" s="24" t="n"/>
@@ -5461,6 +5850,10 @@
         <v/>
       </c>
       <c r="L103" s="39" t="n"/>
+      <c r="N103">
+        <f>IF($B103="","",$C103&amp;"|"&amp;COUNTIF($C$6:$C103,$C103))</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="B104" s="24" t="n"/>
@@ -5477,6 +5870,10 @@
         <v/>
       </c>
       <c r="L104" s="39" t="n"/>
+      <c r="N104">
+        <f>IF($B104="","",$C104&amp;"|"&amp;COUNTIF($C$6:$C104,$C104))</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="B105" s="24" t="n"/>
@@ -5493,6 +5890,10 @@
         <v/>
       </c>
       <c r="L105" s="39" t="n"/>
+      <c r="N105">
+        <f>IF($B105="","",$C105&amp;"|"&amp;COUNTIF($C$6:$C105,$C105))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="B5:L105"/>
@@ -5763,7 +6164,7 @@
         <v/>
       </c>
       <c r="N11">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N11)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N11),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -5809,7 +6210,7 @@
         <v/>
       </c>
       <c r="N12">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N12)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N12),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -5855,7 +6256,7 @@
         <v/>
       </c>
       <c r="N13">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N13)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N13),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -5901,7 +6302,7 @@
         <v/>
       </c>
       <c r="N14">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N14)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N14),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -5947,7 +6348,7 @@
         <v/>
       </c>
       <c r="N15">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N15)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N15),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -5993,7 +6394,7 @@
         <v/>
       </c>
       <c r="N16">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N16)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N16),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6039,7 +6440,7 @@
         <v/>
       </c>
       <c r="N17">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N17)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N17),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6085,7 +6486,7 @@
         <v/>
       </c>
       <c r="N18">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N18)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N18),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6131,7 +6532,7 @@
         <v/>
       </c>
       <c r="N19">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N19)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N19),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6177,7 +6578,7 @@
         <v/>
       </c>
       <c r="N20">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N20)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N20),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6223,7 +6624,7 @@
         <v/>
       </c>
       <c r="N21">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N21)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N21),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6269,7 +6670,7 @@
         <v/>
       </c>
       <c r="N22">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N22)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N22),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6315,7 +6716,7 @@
         <v/>
       </c>
       <c r="N23">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N23)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N23),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6361,7 +6762,7 @@
         <v/>
       </c>
       <c r="N24">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N24)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N24),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6407,7 +6808,7 @@
         <v/>
       </c>
       <c r="N25">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N25)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N25),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6453,7 +6854,7 @@
         <v/>
       </c>
       <c r="N26">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N26)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N26),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6499,7 +6900,7 @@
         <v/>
       </c>
       <c r="N27">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N27)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N27),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6545,7 +6946,7 @@
         <v/>
       </c>
       <c r="N28">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N28)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N28),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6591,7 +6992,7 @@
         <v/>
       </c>
       <c r="N29">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N29)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N29),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6637,7 +7038,7 @@
         <v/>
       </c>
       <c r="N30">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N30)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N30),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6683,7 +7084,7 @@
         <v/>
       </c>
       <c r="N31">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N31)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N31),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6729,7 +7130,7 @@
         <v/>
       </c>
       <c r="N32">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N32)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N32),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6775,7 +7176,7 @@
         <v/>
       </c>
       <c r="N33">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N33)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N33),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6821,7 +7222,7 @@
         <v/>
       </c>
       <c r="N34">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N34)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N34),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6867,7 +7268,7 @@
         <v/>
       </c>
       <c r="N35">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N35)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N35),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6913,7 +7314,7 @@
         <v/>
       </c>
       <c r="N36">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N36)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N36),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -6959,7 +7360,7 @@
         <v/>
       </c>
       <c r="N37">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N37)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N37),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7005,7 +7406,7 @@
         <v/>
       </c>
       <c r="N38">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N38)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N38),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7051,7 +7452,7 @@
         <v/>
       </c>
       <c r="N39">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N39)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N39),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7097,7 +7498,7 @@
         <v/>
       </c>
       <c r="N40">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N40)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N40),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7143,7 +7544,7 @@
         <v/>
       </c>
       <c r="N41">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N41)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N41),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7189,7 +7590,7 @@
         <v/>
       </c>
       <c r="N42">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N42)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N42),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7235,7 +7636,7 @@
         <v/>
       </c>
       <c r="N43">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N43)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N43),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7281,7 +7682,7 @@
         <v/>
       </c>
       <c r="N44">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N44)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N44),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7327,7 +7728,7 @@
         <v/>
       </c>
       <c r="N45">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N45)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N45),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7373,7 +7774,7 @@
         <v/>
       </c>
       <c r="N46">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N46)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N46),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7419,7 +7820,7 @@
         <v/>
       </c>
       <c r="N47">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N47)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N47),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7465,7 +7866,7 @@
         <v/>
       </c>
       <c r="N48">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N48)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N48),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7511,7 +7912,7 @@
         <v/>
       </c>
       <c r="N49">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N49)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N49),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7557,7 +7958,7 @@
         <v/>
       </c>
       <c r="N50">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N50)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N50),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7603,7 +8004,7 @@
         <v/>
       </c>
       <c r="N51">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N51)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N51),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7649,7 +8050,7 @@
         <v/>
       </c>
       <c r="N52">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N52)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N52),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7695,7 +8096,7 @@
         <v/>
       </c>
       <c r="N53">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N53)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N53),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7741,7 +8142,7 @@
         <v/>
       </c>
       <c r="N54">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N54)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N54),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7787,7 +8188,7 @@
         <v/>
       </c>
       <c r="N55">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N55)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N55),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7833,7 +8234,7 @@
         <v/>
       </c>
       <c r="N56">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N56)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N56),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7879,7 +8280,7 @@
         <v/>
       </c>
       <c r="N57">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N57)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N57),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7925,7 +8326,7 @@
         <v/>
       </c>
       <c r="N58">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N58)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N58),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -7971,7 +8372,7 @@
         <v/>
       </c>
       <c r="N59">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N59)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N59),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8017,7 +8418,7 @@
         <v/>
       </c>
       <c r="N60">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N60)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N60),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8063,7 +8464,7 @@
         <v/>
       </c>
       <c r="N61">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N61)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N61),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8109,7 +8510,7 @@
         <v/>
       </c>
       <c r="N62">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N62)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N62),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8155,7 +8556,7 @@
         <v/>
       </c>
       <c r="N63">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N63)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N63),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8201,7 +8602,7 @@
         <v/>
       </c>
       <c r="N64">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N64)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N64),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8247,7 +8648,7 @@
         <v/>
       </c>
       <c r="N65">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N65)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N65),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8293,7 +8694,7 @@
         <v/>
       </c>
       <c r="N66">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N66)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N66),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8339,7 +8740,7 @@
         <v/>
       </c>
       <c r="N67">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N67)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N67),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8385,7 +8786,7 @@
         <v/>
       </c>
       <c r="N68">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N68)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N68),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8431,7 +8832,7 @@
         <v/>
       </c>
       <c r="N69">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N69)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N69),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>
@@ -8477,7 +8878,7 @@
         <v/>
       </c>
       <c r="N70">
-        <f>IF($C$5="","",IFERROR(AGGREGATE(15,6,(ROW(작업!$C$6:$C$105)-5)/((작업!$C$6:$C$105=$C$5)*(작업!$B$6:$B$105&lt;&gt;"")),ROWS($N$11:$N70)),""))</f>
+        <f>IF($C$5="","",IFERROR(MATCH($C$5&amp;"|"&amp;ROWS($N$11:$N70),작업!$N$6:$N$105,0),""))</f>
         <v/>
       </c>
     </row>

</xml_diff>